<commit_message>
Update QA workbook: confirm dashboard charts fixed (DEF-005), DEF-003 config-fixed
</commit_message>
<xml_diff>
--- a/TelemetrixAI_QA_TestExecution_Report.xlsx
+++ b/TelemetrixAI_QA_TestExecution_Report.xlsx
@@ -259,6 +259,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -284,6 +287,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -309,6 +315,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6276,12 +6285,12 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Initially blank (DEF-005: Y-axis fields missing Aggregation wrapper). Fix applied and unit-verified against schema, but not re-confirmed visually by the user after the fix.</t>
-        </is>
-      </c>
-      <c r="I83" s="5" t="inlineStr">
-        <is>
-          <t>PENDING RE-VERIFICATION</t>
+          <t>User-confirmed via screenshot 2026-09-17: line chart shows real data (latency spike visible), column chart shows real anomaly counts per component (cart/checkout/product-catalog), card shows real value (7.95 error_rate_pct). All 3 visuals genuinely rendering.</t>
+        </is>
+      </c>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
@@ -6306,7 +6315,7 @@
       </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>DEF-005 (fixed, unconfirmed visually)</t>
+          <t>DEF-005 (fixed, confirmed)</t>
         </is>
       </c>
     </row>
@@ -6632,7 +6641,7 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Flag's targeting rule returns 'off' unconditionally on both branches of its if/else (a bug in the OTel Demo's own shipped config, not in this project's code) - flag can never actually activate through normal means</t>
+          <t>Targeting rule bug found and fixed (DEF-003): both if/else branches hardcoded to 'off' were corrected so the 'on' branch now actually fires on product_id match. Flag can now activate - not yet exercised with a real capture (no traffic has been driven at the specific targeted product_id).</t>
         </is>
       </c>
       <c r="I88" s="4" t="inlineStr">
@@ -6662,7 +6671,7 @@
       </c>
       <c r="N88" s="2" t="inlineStr">
         <is>
-          <t>DEF-003</t>
+          <t>DEF-003 (config fixed, capture not yet run)</t>
         </is>
       </c>
     </row>
@@ -6977,7 +6986,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Open (third-party/upstream)</t>
+          <t>Fixed (config corrected; real capture against it not yet run)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -6990,7 +6999,11 @@
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Inspect ~/opentelemetry-demo/opentelemetry-demo/src/flagd/demo.flagd.json -&gt; flags.productCatalogFailure.targeting</t>
@@ -7003,7 +7016,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Workaround, not a code fix: directly edit the targeting rule's branches to 'on'/'off' to make it usable, or use a sidecar fault-injection proxy (e.g., Toxiproxy) as already recommended in FINAL_TERM_CONTENT_DRAFT.md Section 10.</t>
+          <t>Workaround, not a code fix: directly edit the targeting rule's branches to 'on'/'off' to make it usable, or use a sidecar fault-injection proxy (e.g., Toxiproxy) as already recommended in FINAL_TERM_CONTENT_DRAFT.md Section 10. UPDATE 2026-09-17: targeting rule if-branch corrected from 'off' to 'on' directly in the demo flagd config (backup kept). Flag can now genuinely activate on the targeted product_id; a real capture exercising it has not yet been run.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr"/>
@@ -7658,6 +7671,8 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
@@ -7745,6 +7760,8 @@
         <v>11</v>
       </c>
     </row>
+    <row r="27"/>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
@@ -7752,6 +7769,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
@@ -7759,6 +7777,41 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
@@ -7766,6 +7819,11 @@
         </is>
       </c>
     </row>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
         <is>

</xml_diff>